<commit_message>
Update the rules engine to the latest version
</commit_message>
<xml_diff>
--- a/resources/templates/report-template.xlsx
+++ b/resources/templates/report-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GerryCampion\Code\cdisc-rules-engine\resources\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamJohnson\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A394FB-97B1-4ED3-8A28-3D9D93F3A0D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0405591-DC0E-4BE6-B2F8-BD5DC0BAE5E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="38670" windowHeight="21150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16275" yWindow="3420" windowWidth="26040" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conformance Details" sheetId="1" r:id="rId1"/>
@@ -152,10 +152,10 @@
     <t>SNOMED Version</t>
   </si>
   <si>
-    <t>TIG Use Case</t>
-  </si>
-  <si>
     <t>LOINC Version</t>
+  </si>
+  <si>
+    <t>TIG Custom Domain Use Case</t>
   </si>
 </sst>
 </file>
@@ -642,34 +642,34 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="82.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="82.42578125" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="13"/>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
@@ -677,7 +677,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>26</v>
       </c>
@@ -685,23 +685,23 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>28</v>
       </c>
       <c r="B8" s="13"/>
     </row>
-    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
@@ -709,32 +709,32 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B13" s="11"/>
     </row>
-    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B14" s="11"/>
     </row>
-    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>34</v>
       </c>
@@ -742,7 +742,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
@@ -750,7 +750,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>37</v>
       </c>
@@ -758,7 +758,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>38</v>
       </c>
@@ -766,7 +766,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>39</v>
       </c>
@@ -774,9 +774,9 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>35</v>
@@ -802,17 +802,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="4" customWidth="1"/>
     <col min="2" max="2" width="36" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="57.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.5546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -832,7 +832,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -840,7 +840,7 @@
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
     </row>
-    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -848,7 +848,7 @@
       <c r="E3" s="5"/>
       <c r="F3" s="5"/>
     </row>
-    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -856,7 +856,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -864,7 +864,7 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -872,7 +872,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -880,7 +880,7 @@
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
     </row>
-    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -888,7 +888,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -896,7 +896,7 @@
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
     </row>
-    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -904,7 +904,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -912,7 +912,7 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
     </row>
-    <row r="12" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -920,7 +920,7 @@
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
@@ -928,7 +928,7 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
     </row>
-    <row r="14" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -936,7 +936,7 @@
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
@@ -944,7 +944,7 @@
       <c r="E15" s="5"/>
       <c r="F15" s="5"/>
     </row>
-    <row r="16" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -952,7 +952,7 @@
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
     </row>
-    <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -960,7 +960,7 @@
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
     </row>
-    <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -968,7 +968,7 @@
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
     </row>
-    <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -976,7 +976,7 @@
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
     </row>
-    <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -984,7 +984,7 @@
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
     </row>
-    <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -992,7 +992,7 @@
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
     </row>
-    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -1000,7 +1000,7 @@
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
     </row>
-    <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -1008,7 +1008,7 @@
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
     </row>
-    <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -1028,16 +1028,16 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" style="4" customWidth="1"/>
     <col min="3" max="3" width="66" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="65.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1054,224 +1054,224 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
     </row>
-    <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
     </row>
-    <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
     </row>
-    <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
     </row>
-    <row r="8" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
     </row>
-    <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
     </row>
-    <row r="11" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
     </row>
-    <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
     </row>
-    <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B15" s="5"/>
       <c r="C15" s="5"/>
     </row>
-    <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
     </row>
-    <row r="17" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
     </row>
-    <row r="18" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
     </row>
-    <row r="19" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
     </row>
-    <row r="20" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
     </row>
-    <row r="21" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
     </row>
-    <row r="22" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
     </row>
-    <row r="23" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
     </row>
-    <row r="24" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
     </row>
-    <row r="25" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
     </row>
-    <row r="26" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
     </row>
-    <row r="27" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
     </row>
-    <row r="28" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
     </row>
-    <row r="29" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
     </row>
-    <row r="30" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
     </row>
-    <row r="31" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
     </row>
-    <row r="32" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
     </row>
-    <row r="33" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
     </row>
-    <row r="34" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
     </row>
-    <row r="35" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
     </row>
-    <row r="36" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
     </row>
-    <row r="37" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
     </row>
-    <row r="38" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
     </row>
-    <row r="39" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
     </row>
-    <row r="40" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
     </row>
-    <row r="41" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
     </row>
-    <row r="42" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
     </row>
-    <row r="43" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
     </row>
-    <row r="44" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
     </row>
-    <row r="45" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
     </row>
-    <row r="46" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
     </row>
-    <row r="47" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
     </row>
-    <row r="48" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
     </row>
-    <row r="49" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
     </row>
-    <row r="50" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B50" s="5"/>
       <c r="C50" s="5"/>
     </row>
-    <row r="51" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
     </row>
-    <row r="52" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
     </row>
-    <row r="53" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
     </row>
-    <row r="54" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
     </row>
-    <row r="55" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
     </row>
-    <row r="56" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
     </row>
@@ -1287,20 +1287,20 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:I147"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.109375" style="4" customWidth="1"/>
-    <col min="2" max="2" width="59.109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="59.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="35.44140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="64.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="64.42578125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1329,738 +1329,738 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="B2" s="6"/>
       <c r="F2" s="6"/>
       <c r="I2" s="5"/>
     </row>
-    <row r="3" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="6"/>
       <c r="F3" s="6"/>
       <c r="I3" s="5"/>
     </row>
-    <row r="4" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
       <c r="F4" s="6"/>
       <c r="I4" s="5"/>
     </row>
-    <row r="5" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
       <c r="F5" s="6"/>
       <c r="I5" s="5"/>
     </row>
-    <row r="6" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
       <c r="F6" s="6"/>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="F7" s="6"/>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="6"/>
       <c r="F8" s="6"/>
     </row>
-    <row r="9" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="F9" s="6"/>
     </row>
-    <row r="10" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="F10" s="6"/>
     </row>
-    <row r="11" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="F11" s="6"/>
     </row>
-    <row r="12" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
       <c r="F12" s="6"/>
     </row>
-    <row r="13" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="F14" s="6"/>
     </row>
-    <row r="15" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="F15" s="6"/>
     </row>
-    <row r="16" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="F16" s="6"/>
     </row>
-    <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="6"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="F18" s="6"/>
     </row>
-    <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="6"/>
       <c r="F19" s="6"/>
     </row>
-    <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="6"/>
       <c r="F20" s="6"/>
     </row>
-    <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" s="6"/>
       <c r="F21" s="6"/>
     </row>
-    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="6"/>
       <c r="F22" s="6"/>
     </row>
-    <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="6"/>
       <c r="F23" s="6"/>
     </row>
-    <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="6"/>
       <c r="F24" s="6"/>
     </row>
-    <row r="25" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>
       <c r="B25" s="6"/>
       <c r="F25" s="6"/>
     </row>
-    <row r="26" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="6"/>
       <c r="F26" s="6"/>
     </row>
-    <row r="27" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="6"/>
       <c r="F27" s="6"/>
     </row>
-    <row r="28" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
       <c r="B28" s="6"/>
       <c r="F28" s="6"/>
     </row>
-    <row r="29" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
       <c r="B29" s="6"/>
       <c r="F29" s="6"/>
     </row>
-    <row r="30" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
       <c r="B30" s="6"/>
       <c r="F30" s="6"/>
     </row>
-    <row r="31" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
       <c r="B31" s="6"/>
       <c r="F31" s="6"/>
     </row>
-    <row r="32" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5"/>
       <c r="B32" s="6"/>
       <c r="F32" s="6"/>
     </row>
-    <row r="33" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
       <c r="B33" s="6"/>
       <c r="F33" s="6"/>
     </row>
-    <row r="34" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
       <c r="B34" s="6"/>
       <c r="F34" s="6"/>
     </row>
-    <row r="35" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="6"/>
       <c r="F35" s="6"/>
     </row>
-    <row r="36" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
       <c r="B36" s="6"/>
       <c r="F36" s="6"/>
     </row>
-    <row r="37" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5"/>
       <c r="B37" s="6"/>
       <c r="F37" s="6"/>
     </row>
-    <row r="38" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
       <c r="B38" s="6"/>
       <c r="F38" s="6"/>
     </row>
-    <row r="39" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
       <c r="B39" s="6"/>
       <c r="F39" s="6"/>
     </row>
-    <row r="40" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
       <c r="B40" s="6"/>
       <c r="F40" s="6"/>
     </row>
-    <row r="41" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
       <c r="B41" s="6"/>
       <c r="F41" s="6"/>
     </row>
-    <row r="42" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
       <c r="B42" s="6"/>
       <c r="F42" s="6"/>
     </row>
-    <row r="43" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
       <c r="B43" s="6"/>
       <c r="F43" s="6"/>
     </row>
-    <row r="44" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
       <c r="B44" s="6"/>
       <c r="F44" s="6"/>
     </row>
-    <row r="45" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5"/>
       <c r="B45" s="6"/>
       <c r="F45" s="6"/>
     </row>
-    <row r="46" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5"/>
       <c r="B46" s="6"/>
       <c r="F46" s="6"/>
     </row>
-    <row r="47" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5"/>
       <c r="B47" s="6"/>
       <c r="F47" s="6"/>
     </row>
-    <row r="48" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5"/>
       <c r="B48" s="6"/>
       <c r="F48" s="6"/>
     </row>
-    <row r="49" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5"/>
       <c r="B49" s="6"/>
       <c r="F49" s="6"/>
     </row>
-    <row r="50" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5"/>
       <c r="B50" s="6"/>
       <c r="F50" s="6"/>
     </row>
-    <row r="51" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5"/>
       <c r="B51" s="6"/>
       <c r="F51" s="6"/>
     </row>
-    <row r="52" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5"/>
       <c r="B52" s="6"/>
       <c r="F52" s="6"/>
     </row>
-    <row r="53" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5"/>
       <c r="B53" s="6"/>
       <c r="F53" s="6"/>
     </row>
-    <row r="54" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5"/>
       <c r="B54" s="6"/>
       <c r="F54" s="6"/>
     </row>
-    <row r="55" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5"/>
       <c r="B55" s="6"/>
       <c r="F55" s="6"/>
     </row>
-    <row r="56" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5"/>
       <c r="B56" s="6"/>
       <c r="F56" s="6"/>
     </row>
-    <row r="57" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5"/>
       <c r="B57" s="6"/>
       <c r="F57" s="6"/>
     </row>
-    <row r="58" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5"/>
       <c r="B58" s="6"/>
       <c r="F58" s="6"/>
     </row>
-    <row r="59" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5"/>
       <c r="B59" s="6"/>
       <c r="F59" s="6"/>
     </row>
-    <row r="60" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5"/>
       <c r="B60" s="6"/>
       <c r="F60" s="6"/>
     </row>
-    <row r="61" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5"/>
       <c r="B61" s="6"/>
       <c r="F61" s="6"/>
     </row>
-    <row r="62" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5"/>
       <c r="B62" s="6"/>
       <c r="F62" s="6"/>
     </row>
-    <row r="63" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5"/>
       <c r="B63" s="6"/>
       <c r="F63" s="6"/>
     </row>
-    <row r="64" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5"/>
       <c r="B64" s="6"/>
       <c r="F64" s="6"/>
     </row>
-    <row r="65" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5"/>
       <c r="B65" s="6"/>
       <c r="F65" s="6"/>
     </row>
-    <row r="66" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5"/>
       <c r="B66" s="6"/>
       <c r="F66" s="6"/>
     </row>
-    <row r="67" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5"/>
       <c r="B67" s="6"/>
       <c r="F67" s="6"/>
     </row>
-    <row r="68" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5"/>
       <c r="B68" s="6"/>
       <c r="F68" s="6"/>
     </row>
-    <row r="69" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5"/>
       <c r="B69" s="6"/>
       <c r="F69" s="6"/>
     </row>
-    <row r="70" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5"/>
       <c r="B70" s="6"/>
       <c r="F70" s="6"/>
     </row>
-    <row r="71" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5"/>
       <c r="B71" s="6"/>
       <c r="F71" s="6"/>
     </row>
-    <row r="72" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5"/>
       <c r="B72" s="6"/>
       <c r="F72" s="6"/>
     </row>
-    <row r="73" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5"/>
       <c r="B73" s="6"/>
       <c r="F73" s="6"/>
     </row>
-    <row r="74" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5"/>
       <c r="B74" s="6"/>
       <c r="F74" s="6"/>
     </row>
-    <row r="75" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5"/>
       <c r="B75" s="6"/>
       <c r="F75" s="6"/>
     </row>
-    <row r="76" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5"/>
       <c r="B76" s="6"/>
       <c r="F76" s="6"/>
     </row>
-    <row r="77" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5"/>
       <c r="B77" s="6"/>
       <c r="F77" s="6"/>
     </row>
-    <row r="78" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5"/>
       <c r="B78" s="6"/>
       <c r="F78" s="6"/>
     </row>
-    <row r="79" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5"/>
       <c r="B79" s="6"/>
       <c r="F79" s="6"/>
     </row>
-    <row r="80" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5"/>
       <c r="B80" s="6"/>
       <c r="F80" s="6"/>
     </row>
-    <row r="81" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5"/>
       <c r="B81" s="6"/>
       <c r="F81" s="6"/>
     </row>
-    <row r="82" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5"/>
       <c r="B82" s="6"/>
       <c r="F82" s="6"/>
     </row>
-    <row r="83" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5"/>
       <c r="B83" s="6"/>
       <c r="F83" s="6"/>
     </row>
-    <row r="84" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5"/>
       <c r="B84" s="6"/>
       <c r="F84" s="6"/>
     </row>
-    <row r="85" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5"/>
       <c r="B85" s="6"/>
       <c r="F85" s="6"/>
     </row>
-    <row r="86" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5"/>
       <c r="B86" s="6"/>
       <c r="F86" s="6"/>
     </row>
-    <row r="87" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5"/>
       <c r="B87" s="6"/>
       <c r="F87" s="6"/>
     </row>
-    <row r="88" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5"/>
       <c r="B88" s="6"/>
       <c r="F88" s="6"/>
     </row>
-    <row r="89" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="5"/>
       <c r="B89" s="6"/>
       <c r="F89" s="6"/>
     </row>
-    <row r="90" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5"/>
       <c r="B90" s="6"/>
       <c r="F90" s="6"/>
     </row>
-    <row r="91" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5"/>
       <c r="B91" s="6"/>
       <c r="F91" s="6"/>
     </row>
-    <row r="92" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5"/>
       <c r="B92" s="6"/>
       <c r="F92" s="6"/>
     </row>
-    <row r="93" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5"/>
       <c r="B93" s="6"/>
       <c r="F93" s="6"/>
     </row>
-    <row r="94" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5"/>
       <c r="B94" s="6"/>
       <c r="F94" s="6"/>
     </row>
-    <row r="95" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5"/>
       <c r="B95" s="6"/>
       <c r="F95" s="6"/>
     </row>
-    <row r="96" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5"/>
       <c r="B96" s="6"/>
       <c r="F96" s="6"/>
     </row>
-    <row r="97" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5"/>
       <c r="B97" s="6"/>
       <c r="F97" s="6"/>
     </row>
-    <row r="98" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5"/>
       <c r="B98" s="6"/>
       <c r="F98" s="6"/>
     </row>
-    <row r="99" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5"/>
       <c r="B99" s="6"/>
       <c r="F99" s="6"/>
     </row>
-    <row r="100" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5"/>
       <c r="B100" s="6"/>
       <c r="F100" s="6"/>
     </row>
-    <row r="101" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5"/>
       <c r="B101" s="6"/>
       <c r="F101" s="6"/>
     </row>
-    <row r="102" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="5"/>
       <c r="B102" s="6"/>
       <c r="F102" s="6"/>
     </row>
-    <row r="103" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5"/>
       <c r="B103" s="6"/>
       <c r="F103" s="6"/>
     </row>
-    <row r="104" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="5"/>
       <c r="B104" s="6"/>
       <c r="F104" s="6"/>
     </row>
-    <row r="105" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5"/>
       <c r="B105" s="6"/>
       <c r="F105" s="6"/>
     </row>
-    <row r="106" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="5"/>
       <c r="B106" s="6"/>
       <c r="F106" s="6"/>
     </row>
-    <row r="107" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="5"/>
       <c r="B107" s="6"/>
       <c r="F107" s="6"/>
     </row>
-    <row r="108" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="5"/>
       <c r="B108" s="6"/>
       <c r="F108" s="6"/>
     </row>
-    <row r="109" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="5"/>
       <c r="B109" s="6"/>
       <c r="F109" s="6"/>
     </row>
-    <row r="110" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="5"/>
       <c r="B110" s="6"/>
       <c r="F110" s="6"/>
     </row>
-    <row r="111" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="5"/>
       <c r="B111" s="6"/>
       <c r="F111" s="6"/>
     </row>
-    <row r="112" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="5"/>
       <c r="B112" s="6"/>
       <c r="F112" s="6"/>
     </row>
-    <row r="113" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="5"/>
       <c r="B113" s="6"/>
       <c r="F113" s="6"/>
     </row>
-    <row r="114" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="5"/>
       <c r="B114" s="6"/>
       <c r="F114" s="6"/>
     </row>
-    <row r="115" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="5"/>
       <c r="B115" s="6"/>
       <c r="F115" s="6"/>
     </row>
-    <row r="116" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="5"/>
       <c r="B116" s="6"/>
       <c r="F116" s="6"/>
     </row>
-    <row r="117" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="5"/>
       <c r="B117" s="6"/>
       <c r="F117" s="6"/>
     </row>
-    <row r="118" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="5"/>
       <c r="B118" s="6"/>
       <c r="F118" s="6"/>
     </row>
-    <row r="119" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="5"/>
       <c r="B119" s="6"/>
       <c r="F119" s="6"/>
     </row>
-    <row r="120" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="5"/>
       <c r="B120" s="6"/>
       <c r="F120" s="6"/>
     </row>
-    <row r="121" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="5"/>
       <c r="B121" s="6"/>
       <c r="F121" s="6"/>
     </row>
-    <row r="122" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="5"/>
       <c r="B122" s="6"/>
       <c r="F122" s="6"/>
     </row>
-    <row r="123" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="5"/>
       <c r="B123" s="6"/>
       <c r="F123" s="6"/>
     </row>
-    <row r="124" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="5"/>
       <c r="B124" s="6"/>
       <c r="F124" s="6"/>
     </row>
-    <row r="125" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="5"/>
       <c r="B125" s="6"/>
       <c r="F125" s="6"/>
     </row>
-    <row r="126" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="5"/>
       <c r="B126" s="6"/>
       <c r="F126" s="6"/>
     </row>
-    <row r="127" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="5"/>
       <c r="B127" s="6"/>
       <c r="F127" s="6"/>
     </row>
-    <row r="128" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="5"/>
       <c r="B128" s="6"/>
       <c r="F128" s="6"/>
     </row>
-    <row r="129" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="5"/>
       <c r="B129" s="6"/>
       <c r="F129" s="6"/>
     </row>
-    <row r="130" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="5"/>
       <c r="B130" s="6"/>
       <c r="F130" s="6"/>
     </row>
-    <row r="131" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="5"/>
       <c r="B131" s="6"/>
       <c r="F131" s="6"/>
     </row>
-    <row r="132" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="5"/>
       <c r="B132" s="6"/>
       <c r="F132" s="6"/>
     </row>
-    <row r="133" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="5"/>
       <c r="B133" s="6"/>
       <c r="F133" s="6"/>
     </row>
-    <row r="134" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="5"/>
       <c r="B134" s="6"/>
       <c r="F134" s="6"/>
     </row>
-    <row r="135" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="5"/>
       <c r="B135" s="6"/>
       <c r="F135" s="6"/>
     </row>
-    <row r="136" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="5"/>
       <c r="B136" s="6"/>
       <c r="F136" s="6"/>
     </row>
-    <row r="137" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="5"/>
       <c r="B137" s="6"/>
       <c r="F137" s="6"/>
     </row>
-    <row r="138" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="5"/>
       <c r="B138" s="6"/>
       <c r="F138" s="6"/>
     </row>
-    <row r="139" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="5"/>
       <c r="B139" s="6"/>
       <c r="F139" s="6"/>
     </row>
-    <row r="140" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="5"/>
       <c r="B140" s="6"/>
       <c r="F140" s="6"/>
     </row>
-    <row r="141" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="5"/>
       <c r="B141" s="6"/>
       <c r="F141" s="6"/>
     </row>
-    <row r="142" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="5"/>
       <c r="B142" s="6"/>
       <c r="F142" s="6"/>
     </row>
-    <row r="143" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5"/>
       <c r="B143" s="6"/>
       <c r="F143" s="6"/>
     </row>
-    <row r="144" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="5"/>
       <c r="B144" s="6"/>
       <c r="F144" s="6"/>
     </row>
-    <row r="145" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="5"/>
       <c r="B145" s="6"/>
       <c r="F145" s="6"/>
     </row>
-    <row r="146" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="5"/>
       <c r="B146" s="6"/>
       <c r="F146" s="6"/>
     </row>
-    <row r="147" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="5"/>
       <c r="B147" s="6"/>
       <c r="F147" s="6"/>
@@ -2077,18 +2077,18 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G197"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.109375" style="4" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" style="4" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" customWidth="1"/>
-    <col min="5" max="5" width="103.44140625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="21.109375" style="4" customWidth="1"/>
-    <col min="7" max="7" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" customWidth="1"/>
+    <col min="5" max="5" width="103.42578125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2109,592 +2109,592 @@
       </c>
       <c r="G1" s="3"/>
     </row>
-    <row r="2" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
     </row>
-    <row r="3" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
     </row>
-    <row r="4" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
     </row>
-    <row r="5" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
     </row>
-    <row r="6" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
     </row>
-    <row r="7" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
     </row>
-    <row r="8" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
     </row>
-    <row r="9" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
     </row>
-    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
     </row>
-    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
     </row>
-    <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
     </row>
-    <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
     </row>
-    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
     </row>
-    <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
     </row>
-    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
     </row>
-    <row r="17" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
     </row>
-    <row r="18" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
     </row>
-    <row r="19" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
     </row>
-    <row r="20" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
     </row>
-    <row r="21" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
     </row>
-    <row r="22" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
     </row>
-    <row r="23" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
     </row>
-    <row r="24" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
     </row>
-    <row r="25" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>
     </row>
-    <row r="26" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
     </row>
-    <row r="27" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
     </row>
-    <row r="28" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
     </row>
-    <row r="29" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
     </row>
-    <row r="30" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
     </row>
-    <row r="31" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
     </row>
-    <row r="32" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5"/>
     </row>
-    <row r="33" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
     </row>
-    <row r="34" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
     </row>
-    <row r="35" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
     </row>
-    <row r="36" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
     </row>
-    <row r="37" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5"/>
     </row>
-    <row r="38" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
     </row>
-    <row r="39" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
     </row>
-    <row r="40" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
     </row>
-    <row r="41" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
     </row>
-    <row r="42" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
     </row>
-    <row r="43" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
     </row>
-    <row r="44" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
     </row>
-    <row r="45" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5"/>
     </row>
-    <row r="46" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5"/>
     </row>
-    <row r="47" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5"/>
     </row>
-    <row r="48" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5"/>
     </row>
-    <row r="49" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5"/>
     </row>
-    <row r="50" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5"/>
     </row>
-    <row r="51" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5"/>
     </row>
-    <row r="52" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5"/>
     </row>
-    <row r="53" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5"/>
     </row>
-    <row r="54" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5"/>
     </row>
-    <row r="55" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5"/>
     </row>
-    <row r="56" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5"/>
     </row>
-    <row r="57" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5"/>
     </row>
-    <row r="58" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5"/>
     </row>
-    <row r="59" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5"/>
     </row>
-    <row r="60" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5"/>
     </row>
-    <row r="61" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5"/>
     </row>
-    <row r="62" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5"/>
     </row>
-    <row r="63" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5"/>
     </row>
-    <row r="64" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5"/>
     </row>
-    <row r="65" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5"/>
     </row>
-    <row r="66" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5"/>
     </row>
-    <row r="67" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5"/>
     </row>
-    <row r="68" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5"/>
     </row>
-    <row r="69" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5"/>
     </row>
-    <row r="70" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5"/>
     </row>
-    <row r="71" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5"/>
     </row>
-    <row r="72" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5"/>
     </row>
-    <row r="73" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5"/>
     </row>
-    <row r="74" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5"/>
     </row>
-    <row r="75" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5"/>
     </row>
-    <row r="76" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5"/>
     </row>
-    <row r="77" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5"/>
     </row>
-    <row r="78" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5"/>
     </row>
-    <row r="79" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5"/>
     </row>
-    <row r="80" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5"/>
     </row>
-    <row r="81" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5"/>
     </row>
-    <row r="82" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5"/>
     </row>
-    <row r="83" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5"/>
     </row>
-    <row r="84" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5"/>
     </row>
-    <row r="85" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5"/>
     </row>
-    <row r="86" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5"/>
     </row>
-    <row r="87" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5"/>
     </row>
-    <row r="88" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5"/>
     </row>
-    <row r="89" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="5"/>
     </row>
-    <row r="90" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5"/>
     </row>
-    <row r="91" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5"/>
     </row>
-    <row r="92" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5"/>
     </row>
-    <row r="93" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5"/>
     </row>
-    <row r="94" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5"/>
     </row>
-    <row r="95" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5"/>
     </row>
-    <row r="96" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5"/>
     </row>
-    <row r="97" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5"/>
     </row>
-    <row r="98" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5"/>
     </row>
-    <row r="99" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5"/>
     </row>
-    <row r="100" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5"/>
     </row>
-    <row r="101" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5"/>
     </row>
-    <row r="102" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="5"/>
     </row>
-    <row r="103" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="5"/>
     </row>
-    <row r="104" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="5"/>
     </row>
-    <row r="105" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="5"/>
     </row>
-    <row r="106" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="5"/>
     </row>
-    <row r="107" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="5"/>
     </row>
-    <row r="108" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="5"/>
     </row>
-    <row r="109" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="5"/>
     </row>
-    <row r="110" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="5"/>
     </row>
-    <row r="111" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="5"/>
     </row>
-    <row r="112" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="5"/>
     </row>
-    <row r="113" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="5"/>
     </row>
-    <row r="114" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="5"/>
     </row>
-    <row r="115" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="5"/>
     </row>
-    <row r="116" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="5"/>
     </row>
-    <row r="117" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="5"/>
     </row>
-    <row r="118" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="5"/>
     </row>
-    <row r="119" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="5"/>
     </row>
-    <row r="120" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="5"/>
     </row>
-    <row r="121" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="5"/>
     </row>
-    <row r="122" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="5"/>
     </row>
-    <row r="123" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="5"/>
     </row>
-    <row r="124" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="5"/>
     </row>
-    <row r="125" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="5"/>
     </row>
-    <row r="126" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="5"/>
     </row>
-    <row r="127" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="5"/>
     </row>
-    <row r="128" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="5"/>
     </row>
-    <row r="129" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="5"/>
     </row>
-    <row r="130" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="5"/>
     </row>
-    <row r="131" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="5"/>
     </row>
-    <row r="132" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="5"/>
     </row>
-    <row r="133" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="5"/>
     </row>
-    <row r="134" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="5"/>
     </row>
-    <row r="135" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="5"/>
     </row>
-    <row r="136" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="5"/>
     </row>
-    <row r="137" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="5"/>
     </row>
-    <row r="138" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="5"/>
     </row>
-    <row r="139" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="5"/>
     </row>
-    <row r="140" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="5"/>
     </row>
-    <row r="141" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="5"/>
     </row>
-    <row r="142" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="5"/>
     </row>
-    <row r="143" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="5"/>
     </row>
-    <row r="144" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="5"/>
     </row>
-    <row r="145" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="5"/>
     </row>
-    <row r="146" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="5"/>
     </row>
-    <row r="147" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="5"/>
     </row>
-    <row r="148" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="5"/>
     </row>
-    <row r="149" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="5"/>
     </row>
-    <row r="150" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="5"/>
     </row>
-    <row r="151" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="5"/>
     </row>
-    <row r="152" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="5"/>
     </row>
-    <row r="153" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="5"/>
     </row>
-    <row r="154" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="5"/>
     </row>
-    <row r="155" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="5"/>
     </row>
-    <row r="156" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="5"/>
     </row>
-    <row r="157" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="5"/>
     </row>
-    <row r="158" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="5"/>
     </row>
-    <row r="159" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="5"/>
     </row>
-    <row r="160" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="5"/>
     </row>
-    <row r="161" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="5"/>
     </row>
-    <row r="162" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="5"/>
     </row>
-    <row r="163" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="5"/>
     </row>
-    <row r="164" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="5"/>
     </row>
-    <row r="165" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="5"/>
     </row>
-    <row r="166" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="5"/>
     </row>
-    <row r="167" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="5"/>
     </row>
-    <row r="168" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="5"/>
     </row>
-    <row r="169" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="5"/>
     </row>
-    <row r="170" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="5"/>
     </row>
-    <row r="171" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="5"/>
     </row>
-    <row r="172" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="5"/>
     </row>
-    <row r="173" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="5"/>
     </row>
-    <row r="174" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="5"/>
     </row>
-    <row r="175" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="5"/>
     </row>
-    <row r="176" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="5"/>
     </row>
-    <row r="177" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="5"/>
     </row>
-    <row r="178" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="5"/>
     </row>
-    <row r="179" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="5"/>
     </row>
-    <row r="180" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="5"/>
     </row>
-    <row r="181" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="5"/>
     </row>
-    <row r="182" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="5"/>
     </row>
-    <row r="183" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="5"/>
     </row>
-    <row r="184" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="5"/>
     </row>
-    <row r="185" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="5"/>
     </row>
-    <row r="186" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="5"/>
     </row>
-    <row r="187" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="5"/>
     </row>
-    <row r="188" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="5"/>
     </row>
-    <row r="189" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="5"/>
     </row>
-    <row r="190" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="5"/>
     </row>
-    <row r="191" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="5"/>
     </row>
-    <row r="192" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="5"/>
     </row>
-    <row r="193" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="5"/>
     </row>
-    <row r="194" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="5"/>
     </row>
-    <row r="195" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="5"/>
     </row>
-    <row r="196" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="5"/>
     </row>
-    <row r="197" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="5"/>
     </row>
   </sheetData>

</xml_diff>